<commit_message>
Update CP-FGW-L0-MVAC panel schedule to latest MVAC equipment list
- Rebuild panel schedule (R2) per latest cooling load & fan schedule:
  45x 3.7 kW wall fans, EF D-002, 14 Daikin split units, small 1-ph fans
- 4 busbar rows x 17 ways (65 circuits + 3 spare), 1-ph loads balanced on R/S/T
- Breakers, cables and DOL starters resized; Pt/Pact and incomer updated
- Fix Excel power consumption unit (WATT -> kW), EF D-101/D-102 rooms

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FfhKtLLxtUCbEHbugUZExH
</commit_message>
<xml_diff>
--- a/exports/HBE_Cooling_Load_and_Fan_Schedule.xlsx
+++ b/exports/HBE_Cooling_Load_and_Fan_Schedule.xlsx
@@ -689,7 +689,7 @@
       </c>
       <c r="Q7" s="4" t="inlineStr">
         <is>
-          <t>POWER CONSUMPTION (WATT)</t>
+          <t>POWER CONSUMPTION (kW)</t>
         </is>
       </c>
       <c r="R7" s="9" t="n"/>
@@ -2096,7 +2096,7 @@
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>EF D-102</t>
+          <t>EF D-101</t>
         </is>
       </c>
       <c r="B10" s="10" t="n"/>
@@ -2142,7 +2142,7 @@
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>EF D-101</t>
+          <t>EF D-102</t>
         </is>
       </c>
       <c r="B11" s="10" t="n"/>

</xml_diff>